<commit_message>
Actualiza histórico prdemcad + csv
</commit_message>
<xml_diff>
--- a/Historico_prdemcad.xlsx
+++ b/Historico_prdemcad.xlsx
@@ -80188,7 +80188,7 @@
         <v>2</v>
       </c>
       <c r="G2954" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2955">
@@ -80215,7 +80215,7 @@
         <v>2</v>
       </c>
       <c r="G2955" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2956">
@@ -80242,7 +80242,7 @@
         <v>2</v>
       </c>
       <c r="G2956" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2957">
@@ -80269,7 +80269,7 @@
         <v>2</v>
       </c>
       <c r="G2957" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2958">
@@ -80296,7 +80296,7 @@
         <v>2</v>
       </c>
       <c r="G2958" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2959">
@@ -80323,7 +80323,7 @@
         <v>2</v>
       </c>
       <c r="G2959" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2960">
@@ -80350,7 +80350,7 @@
         <v>2</v>
       </c>
       <c r="G2960" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2961">
@@ -80377,7 +80377,7 @@
         <v>2</v>
       </c>
       <c r="G2961" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2962">
@@ -80404,7 +80404,7 @@
         <v>2</v>
       </c>
       <c r="G2962" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2963">
@@ -80431,7 +80431,7 @@
         <v>2</v>
       </c>
       <c r="G2963" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2964">
@@ -80458,7 +80458,7 @@
         <v>2</v>
       </c>
       <c r="G2964" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2965">
@@ -80485,7 +80485,7 @@
         <v>2</v>
       </c>
       <c r="G2965" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2966">
@@ -80512,7 +80512,7 @@
         <v>2</v>
       </c>
       <c r="G2966" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2967">
@@ -80539,7 +80539,7 @@
         <v>2</v>
       </c>
       <c r="G2967" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2968">
@@ -80566,7 +80566,7 @@
         <v>2</v>
       </c>
       <c r="G2968" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2969">
@@ -80593,7 +80593,7 @@
         <v>2</v>
       </c>
       <c r="G2969" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2970">
@@ -80620,7 +80620,7 @@
         <v>2</v>
       </c>
       <c r="G2970" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2971">
@@ -80647,7 +80647,7 @@
         <v>2</v>
       </c>
       <c r="G2971" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2972">
@@ -80674,7 +80674,7 @@
         <v>2</v>
       </c>
       <c r="G2972" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2973">
@@ -80701,7 +80701,7 @@
         <v>2</v>
       </c>
       <c r="G2973" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2974">
@@ -80728,7 +80728,7 @@
         <v>2</v>
       </c>
       <c r="G2974" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2975">
@@ -80755,7 +80755,7 @@
         <v>2</v>
       </c>
       <c r="G2975" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2976">
@@ -80782,7 +80782,7 @@
         <v>2</v>
       </c>
       <c r="G2976" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2977">
@@ -80809,7 +80809,7 @@
         <v>2</v>
       </c>
       <c r="G2977" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2978">
@@ -80836,7 +80836,7 @@
         <v>2</v>
       </c>
       <c r="G2978" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2979">
@@ -80863,7 +80863,7 @@
         <v>2</v>
       </c>
       <c r="G2979" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2980">
@@ -80890,7 +80890,7 @@
         <v>2</v>
       </c>
       <c r="G2980" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2981">
@@ -80917,7 +80917,7 @@
         <v>2</v>
       </c>
       <c r="G2981" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2982">
@@ -80944,7 +80944,7 @@
         <v>2</v>
       </c>
       <c r="G2982" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2983">
@@ -80971,7 +80971,7 @@
         <v>2</v>
       </c>
       <c r="G2983" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2984">
@@ -80998,7 +80998,7 @@
         <v>2</v>
       </c>
       <c r="G2984" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2985">
@@ -81025,7 +81025,7 @@
         <v>2</v>
       </c>
       <c r="G2985" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2986">
@@ -81052,7 +81052,7 @@
         <v>2</v>
       </c>
       <c r="G2986" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2987">
@@ -81079,7 +81079,7 @@
         <v>2</v>
       </c>
       <c r="G2987" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2988">
@@ -81106,7 +81106,7 @@
         <v>2</v>
       </c>
       <c r="G2988" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2989">
@@ -81133,7 +81133,7 @@
         <v>2</v>
       </c>
       <c r="G2989" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2990">
@@ -81160,7 +81160,7 @@
         <v>2</v>
       </c>
       <c r="G2990" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2991">
@@ -81187,7 +81187,7 @@
         <v>2</v>
       </c>
       <c r="G2991" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2992">
@@ -81214,7 +81214,7 @@
         <v>2</v>
       </c>
       <c r="G2992" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2993">
@@ -81241,7 +81241,7 @@
         <v>2</v>
       </c>
       <c r="G2993" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2994">
@@ -81268,7 +81268,7 @@
         <v>2</v>
       </c>
       <c r="G2994" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2995">
@@ -81295,7 +81295,7 @@
         <v>2</v>
       </c>
       <c r="G2995" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2996">
@@ -81322,7 +81322,7 @@
         <v>2</v>
       </c>
       <c r="G2996" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2997">
@@ -81349,7 +81349,7 @@
         <v>2</v>
       </c>
       <c r="G2997" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2998">
@@ -81376,7 +81376,7 @@
         <v>2</v>
       </c>
       <c r="G2998" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="2999">
@@ -81403,7 +81403,7 @@
         <v>2</v>
       </c>
       <c r="G2999" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3000">
@@ -81430,7 +81430,7 @@
         <v>2</v>
       </c>
       <c r="G3000" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3001">
@@ -81457,7 +81457,7 @@
         <v>2</v>
       </c>
       <c r="G3001" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3002">
@@ -81484,7 +81484,7 @@
         <v>2</v>
       </c>
       <c r="G3002" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3003">
@@ -81511,7 +81511,7 @@
         <v>2</v>
       </c>
       <c r="G3003" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3004">
@@ -81538,7 +81538,7 @@
         <v>2</v>
       </c>
       <c r="G3004" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3005">
@@ -81565,7 +81565,7 @@
         <v>2</v>
       </c>
       <c r="G3005" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3006">
@@ -81592,7 +81592,7 @@
         <v>2</v>
       </c>
       <c r="G3006" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3007">
@@ -81619,7 +81619,7 @@
         <v>2</v>
       </c>
       <c r="G3007" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3008">
@@ -81646,7 +81646,7 @@
         <v>2</v>
       </c>
       <c r="G3008" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3009">
@@ -81673,7 +81673,7 @@
         <v>2</v>
       </c>
       <c r="G3009" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3010">
@@ -81700,7 +81700,7 @@
         <v>2</v>
       </c>
       <c r="G3010" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3011">
@@ -81727,7 +81727,7 @@
         <v>2</v>
       </c>
       <c r="G3011" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3012">
@@ -81754,7 +81754,7 @@
         <v>2</v>
       </c>
       <c r="G3012" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3013">
@@ -81781,7 +81781,7 @@
         <v>2</v>
       </c>
       <c r="G3013" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3014">
@@ -81808,7 +81808,7 @@
         <v>2</v>
       </c>
       <c r="G3014" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3015">
@@ -81835,7 +81835,7 @@
         <v>2</v>
       </c>
       <c r="G3015" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3016">
@@ -81862,7 +81862,7 @@
         <v>2</v>
       </c>
       <c r="G3016" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3017">
@@ -81889,7 +81889,7 @@
         <v>2</v>
       </c>
       <c r="G3017" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3018">
@@ -81916,7 +81916,7 @@
         <v>2</v>
       </c>
       <c r="G3018" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3019">
@@ -81943,7 +81943,7 @@
         <v>2</v>
       </c>
       <c r="G3019" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3020">
@@ -81970,7 +81970,7 @@
         <v>2</v>
       </c>
       <c r="G3020" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3021">
@@ -81997,7 +81997,7 @@
         <v>2</v>
       </c>
       <c r="G3021" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3022">
@@ -82024,7 +82024,7 @@
         <v>2</v>
       </c>
       <c r="G3022" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3023">
@@ -82051,7 +82051,7 @@
         <v>2</v>
       </c>
       <c r="G3023" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3024">
@@ -82078,7 +82078,7 @@
         <v>2</v>
       </c>
       <c r="G3024" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3025">
@@ -82105,7 +82105,7 @@
         <v>2</v>
       </c>
       <c r="G3025" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3026">
@@ -82132,7 +82132,7 @@
         <v>2</v>
       </c>
       <c r="G3026" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3027">
@@ -82159,7 +82159,7 @@
         <v>2</v>
       </c>
       <c r="G3027" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3028">
@@ -82186,7 +82186,7 @@
         <v>2</v>
       </c>
       <c r="G3028" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3029">
@@ -82213,7 +82213,7 @@
         <v>2</v>
       </c>
       <c r="G3029" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3030">
@@ -82240,7 +82240,7 @@
         <v>2</v>
       </c>
       <c r="G3030" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3031">
@@ -82267,7 +82267,7 @@
         <v>2</v>
       </c>
       <c r="G3031" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3032">
@@ -82294,7 +82294,7 @@
         <v>2</v>
       </c>
       <c r="G3032" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3033">
@@ -82321,7 +82321,7 @@
         <v>2</v>
       </c>
       <c r="G3033" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3034">
@@ -82348,7 +82348,7 @@
         <v>2</v>
       </c>
       <c r="G3034" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3035">
@@ -82375,7 +82375,7 @@
         <v>2</v>
       </c>
       <c r="G3035" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3036">
@@ -82402,7 +82402,7 @@
         <v>2</v>
       </c>
       <c r="G3036" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3037">
@@ -82429,7 +82429,7 @@
         <v>2</v>
       </c>
       <c r="G3037" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3038">
@@ -82456,7 +82456,7 @@
         <v>2</v>
       </c>
       <c r="G3038" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3039">
@@ -82483,7 +82483,7 @@
         <v>2</v>
       </c>
       <c r="G3039" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3040">
@@ -82510,7 +82510,7 @@
         <v>2</v>
       </c>
       <c r="G3040" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3041">
@@ -82537,7 +82537,7 @@
         <v>2</v>
       </c>
       <c r="G3041" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3042">
@@ -82564,7 +82564,7 @@
         <v>2</v>
       </c>
       <c r="G3042" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3043">
@@ -82591,7 +82591,7 @@
         <v>2</v>
       </c>
       <c r="G3043" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3044">
@@ -82618,7 +82618,7 @@
         <v>2</v>
       </c>
       <c r="G3044" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3045">
@@ -82645,7 +82645,7 @@
         <v>2</v>
       </c>
       <c r="G3045" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3046">
@@ -82672,7 +82672,7 @@
         <v>2</v>
       </c>
       <c r="G3046" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3047">
@@ -82699,7 +82699,7 @@
         <v>2</v>
       </c>
       <c r="G3047" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3048">
@@ -82726,7 +82726,7 @@
         <v>2</v>
       </c>
       <c r="G3048" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3049">
@@ -82753,7 +82753,7 @@
         <v>2</v>
       </c>
       <c r="G3049" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3050">
@@ -82780,7 +82780,7 @@
         <v>2</v>
       </c>
       <c r="G3050" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3051">
@@ -82807,7 +82807,7 @@
         <v>2</v>
       </c>
       <c r="G3051" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3052">
@@ -82834,7 +82834,7 @@
         <v>2</v>
       </c>
       <c r="G3052" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3053">
@@ -82861,7 +82861,7 @@
         <v>2</v>
       </c>
       <c r="G3053" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3054">
@@ -82888,7 +82888,7 @@
         <v>2</v>
       </c>
       <c r="G3054" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3055">
@@ -82915,7 +82915,7 @@
         <v>2</v>
       </c>
       <c r="G3055" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3056">
@@ -82942,7 +82942,7 @@
         <v>2</v>
       </c>
       <c r="G3056" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3057">
@@ -82969,7 +82969,7 @@
         <v>2</v>
       </c>
       <c r="G3057" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3058">
@@ -82996,7 +82996,7 @@
         <v>2</v>
       </c>
       <c r="G3058" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3059">
@@ -83023,7 +83023,7 @@
         <v>2</v>
       </c>
       <c r="G3059" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3060">
@@ -83050,7 +83050,7 @@
         <v>2</v>
       </c>
       <c r="G3060" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3061">
@@ -83077,7 +83077,7 @@
         <v>2</v>
       </c>
       <c r="G3061" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3062">
@@ -83104,7 +83104,7 @@
         <v>2</v>
       </c>
       <c r="G3062" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3063">
@@ -83131,7 +83131,7 @@
         <v>2</v>
       </c>
       <c r="G3063" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3064">
@@ -83158,7 +83158,7 @@
         <v>2</v>
       </c>
       <c r="G3064" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3065">
@@ -83185,7 +83185,7 @@
         <v>2</v>
       </c>
       <c r="G3065" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3066">
@@ -83212,7 +83212,7 @@
         <v>2</v>
       </c>
       <c r="G3066" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3067">
@@ -83239,7 +83239,7 @@
         <v>2</v>
       </c>
       <c r="G3067" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3068">
@@ -83266,7 +83266,7 @@
         <v>2</v>
       </c>
       <c r="G3068" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3069">
@@ -83293,7 +83293,7 @@
         <v>2</v>
       </c>
       <c r="G3069" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3070">
@@ -83320,7 +83320,7 @@
         <v>2</v>
       </c>
       <c r="G3070" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3071">
@@ -83347,7 +83347,7 @@
         <v>2</v>
       </c>
       <c r="G3071" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3072">
@@ -83374,7 +83374,7 @@
         <v>2</v>
       </c>
       <c r="G3072" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3073">
@@ -83401,7 +83401,7 @@
         <v>2</v>
       </c>
       <c r="G3073" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3074">
@@ -83428,7 +83428,7 @@
         <v>2</v>
       </c>
       <c r="G3074" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3075">
@@ -83455,7 +83455,7 @@
         <v>2</v>
       </c>
       <c r="G3075" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3076">
@@ -83482,7 +83482,7 @@
         <v>2</v>
       </c>
       <c r="G3076" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3077">
@@ -83509,7 +83509,7 @@
         <v>2</v>
       </c>
       <c r="G3077" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3078">
@@ -83536,7 +83536,7 @@
         <v>2</v>
       </c>
       <c r="G3078" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3079">
@@ -83563,7 +83563,7 @@
         <v>2</v>
       </c>
       <c r="G3079" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3080">
@@ -83590,7 +83590,7 @@
         <v>2</v>
       </c>
       <c r="G3080" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3081">
@@ -83617,7 +83617,7 @@
         <v>2</v>
       </c>
       <c r="G3081" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3082">
@@ -83644,7 +83644,7 @@
         <v>2</v>
       </c>
       <c r="G3082" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3083">
@@ -83671,7 +83671,7 @@
         <v>2</v>
       </c>
       <c r="G3083" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3084">
@@ -83698,7 +83698,7 @@
         <v>2</v>
       </c>
       <c r="G3084" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3085">
@@ -83725,7 +83725,7 @@
         <v>2</v>
       </c>
       <c r="G3085" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3086">
@@ -83752,7 +83752,7 @@
         <v>2</v>
       </c>
       <c r="G3086" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3087">
@@ -83779,7 +83779,7 @@
         <v>2</v>
       </c>
       <c r="G3087" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3088">
@@ -83806,7 +83806,7 @@
         <v>2</v>
       </c>
       <c r="G3088" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3089">
@@ -83833,7 +83833,7 @@
         <v>2</v>
       </c>
       <c r="G3089" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3090">
@@ -83860,7 +83860,7 @@
         <v>2</v>
       </c>
       <c r="G3090" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3091">
@@ -83887,7 +83887,7 @@
         <v>2</v>
       </c>
       <c r="G3091" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3092">
@@ -83914,7 +83914,7 @@
         <v>2</v>
       </c>
       <c r="G3092" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3093">
@@ -83941,7 +83941,7 @@
         <v>2</v>
       </c>
       <c r="G3093" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3094">
@@ -83968,7 +83968,7 @@
         <v>2</v>
       </c>
       <c r="G3094" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3095">
@@ -83995,7 +83995,7 @@
         <v>2</v>
       </c>
       <c r="G3095" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3096">
@@ -84022,7 +84022,7 @@
         <v>2</v>
       </c>
       <c r="G3096" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3097">
@@ -84049,7 +84049,7 @@
         <v>2</v>
       </c>
       <c r="G3097" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3098">
@@ -84076,7 +84076,7 @@
         <v>2</v>
       </c>
       <c r="G3098" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3099">
@@ -84103,7 +84103,7 @@
         <v>2</v>
       </c>
       <c r="G3099" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3100">
@@ -84130,7 +84130,7 @@
         <v>2</v>
       </c>
       <c r="G3100" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3101">
@@ -84157,7 +84157,7 @@
         <v>2</v>
       </c>
       <c r="G3101" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3102">
@@ -84184,7 +84184,7 @@
         <v>2</v>
       </c>
       <c r="G3102" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3103">
@@ -84211,7 +84211,7 @@
         <v>2</v>
       </c>
       <c r="G3103" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3104">
@@ -84238,7 +84238,7 @@
         <v>2</v>
       </c>
       <c r="G3104" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3105">
@@ -84265,7 +84265,7 @@
         <v>2</v>
       </c>
       <c r="G3105" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3106">
@@ -84292,7 +84292,7 @@
         <v>2</v>
       </c>
       <c r="G3106" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3107">
@@ -84319,7 +84319,7 @@
         <v>2</v>
       </c>
       <c r="G3107" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3108">
@@ -84346,7 +84346,7 @@
         <v>2</v>
       </c>
       <c r="G3108" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3109">
@@ -84373,7 +84373,7 @@
         <v>2</v>
       </c>
       <c r="G3109" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3110">
@@ -84400,7 +84400,7 @@
         <v>2</v>
       </c>
       <c r="G3110" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3111">
@@ -84427,7 +84427,7 @@
         <v>2</v>
       </c>
       <c r="G3111" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3112">
@@ -84454,7 +84454,7 @@
         <v>2</v>
       </c>
       <c r="G3112" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3113">
@@ -84481,7 +84481,7 @@
         <v>2</v>
       </c>
       <c r="G3113" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3114">
@@ -84508,7 +84508,7 @@
         <v>2</v>
       </c>
       <c r="G3114" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3115">
@@ -84535,7 +84535,7 @@
         <v>2</v>
       </c>
       <c r="G3115" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3116">
@@ -84562,7 +84562,7 @@
         <v>2</v>
       </c>
       <c r="G3116" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3117">
@@ -84589,7 +84589,7 @@
         <v>2</v>
       </c>
       <c r="G3117" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3118">
@@ -84616,7 +84616,7 @@
         <v>2</v>
       </c>
       <c r="G3118" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3119">
@@ -84643,7 +84643,7 @@
         <v>2</v>
       </c>
       <c r="G3119" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3120">
@@ -84670,7 +84670,7 @@
         <v>2</v>
       </c>
       <c r="G3120" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3121">
@@ -84697,7 +84697,7 @@
         <v>2</v>
       </c>
       <c r="G3121" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3122">
@@ -84724,7 +84724,7 @@
         <v>2</v>
       </c>
       <c r="G3122" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3123">
@@ -84751,7 +84751,7 @@
         <v>2</v>
       </c>
       <c r="G3123" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3124">
@@ -84778,7 +84778,7 @@
         <v>2</v>
       </c>
       <c r="G3124" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3125">
@@ -84805,7 +84805,7 @@
         <v>2</v>
       </c>
       <c r="G3125" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3126">
@@ -84832,7 +84832,7 @@
         <v>2</v>
       </c>
       <c r="G3126" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3127">
@@ -84859,7 +84859,7 @@
         <v>2</v>
       </c>
       <c r="G3127" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3128">
@@ -84886,7 +84886,7 @@
         <v>2</v>
       </c>
       <c r="G3128" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3129">
@@ -84913,7 +84913,7 @@
         <v>2</v>
       </c>
       <c r="G3129" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3130">
@@ -84940,7 +84940,7 @@
         <v>2</v>
       </c>
       <c r="G3130" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3131">
@@ -84967,7 +84967,7 @@
         <v>2</v>
       </c>
       <c r="G3131" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3132">
@@ -84994,7 +84994,7 @@
         <v>2</v>
       </c>
       <c r="G3132" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3133">
@@ -85021,7 +85021,7 @@
         <v>2</v>
       </c>
       <c r="G3133" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3134">
@@ -85048,7 +85048,7 @@
         <v>2</v>
       </c>
       <c r="G3134" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3135">
@@ -85075,7 +85075,7 @@
         <v>2</v>
       </c>
       <c r="G3135" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3136">
@@ -85102,7 +85102,7 @@
         <v>2</v>
       </c>
       <c r="G3136" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3137">
@@ -85129,7 +85129,7 @@
         <v>2</v>
       </c>
       <c r="G3137" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3138">
@@ -85156,7 +85156,7 @@
         <v>2</v>
       </c>
       <c r="G3138" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3139">
@@ -85183,7 +85183,7 @@
         <v>2</v>
       </c>
       <c r="G3139" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3140">
@@ -85210,7 +85210,7 @@
         <v>2</v>
       </c>
       <c r="G3140" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3141">
@@ -85237,7 +85237,7 @@
         <v>2</v>
       </c>
       <c r="G3141" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3142">
@@ -85264,7 +85264,7 @@
         <v>2</v>
       </c>
       <c r="G3142" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3143">
@@ -85291,7 +85291,7 @@
         <v>2</v>
       </c>
       <c r="G3143" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3144">
@@ -85318,7 +85318,7 @@
         <v>2</v>
       </c>
       <c r="G3144" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3145">
@@ -85345,7 +85345,7 @@
         <v>2</v>
       </c>
       <c r="G3145" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3146">
@@ -85372,7 +85372,7 @@
         <v>2</v>
       </c>
       <c r="G3146" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3147">
@@ -85399,7 +85399,7 @@
         <v>2</v>
       </c>
       <c r="G3147" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3148">
@@ -85426,7 +85426,7 @@
         <v>2</v>
       </c>
       <c r="G3148" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3149">
@@ -85453,7 +85453,7 @@
         <v>2</v>
       </c>
       <c r="G3149" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3150">
@@ -85480,7 +85480,7 @@
         <v>2</v>
       </c>
       <c r="G3150" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3151">
@@ -85507,7 +85507,7 @@
         <v>2</v>
       </c>
       <c r="G3151" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3152">
@@ -85534,7 +85534,7 @@
         <v>2</v>
       </c>
       <c r="G3152" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3153">
@@ -85561,7 +85561,7 @@
         <v>2</v>
       </c>
       <c r="G3153" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3154">
@@ -85588,7 +85588,7 @@
         <v>2</v>
       </c>
       <c r="G3154" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3155">
@@ -85615,7 +85615,7 @@
         <v>2</v>
       </c>
       <c r="G3155" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3156">
@@ -85642,7 +85642,7 @@
         <v>2</v>
       </c>
       <c r="G3156" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3157">
@@ -85669,7 +85669,7 @@
         <v>2</v>
       </c>
       <c r="G3157" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3158">
@@ -85696,7 +85696,7 @@
         <v>2</v>
       </c>
       <c r="G3158" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3159">
@@ -85723,7 +85723,7 @@
         <v>2</v>
       </c>
       <c r="G3159" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3160">
@@ -85750,7 +85750,7 @@
         <v>2</v>
       </c>
       <c r="G3160" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3161">
@@ -85777,7 +85777,7 @@
         <v>2</v>
       </c>
       <c r="G3161" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3162">
@@ -85804,7 +85804,7 @@
         <v>2</v>
       </c>
       <c r="G3162" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3163">
@@ -85831,7 +85831,7 @@
         <v>2</v>
       </c>
       <c r="G3163" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3164">
@@ -85858,7 +85858,7 @@
         <v>2</v>
       </c>
       <c r="G3164" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3165">
@@ -85885,7 +85885,7 @@
         <v>2</v>
       </c>
       <c r="G3165" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3166">
@@ -85912,7 +85912,7 @@
         <v>2</v>
       </c>
       <c r="G3166" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3167">
@@ -85939,7 +85939,7 @@
         <v>2</v>
       </c>
       <c r="G3167" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3168">
@@ -85966,7 +85966,7 @@
         <v>2</v>
       </c>
       <c r="G3168" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3169">
@@ -85993,7 +85993,7 @@
         <v>2</v>
       </c>
       <c r="G3169" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3170">
@@ -86020,7 +86020,7 @@
         <v>2</v>
       </c>
       <c r="G3170" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3171">
@@ -86047,7 +86047,7 @@
         <v>2</v>
       </c>
       <c r="G3171" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3172">
@@ -86074,7 +86074,7 @@
         <v>2</v>
       </c>
       <c r="G3172" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3173">
@@ -86101,7 +86101,7 @@
         <v>2</v>
       </c>
       <c r="G3173" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3174">
@@ -86128,7 +86128,7 @@
         <v>2</v>
       </c>
       <c r="G3174" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3175">
@@ -86155,7 +86155,7 @@
         <v>2</v>
       </c>
       <c r="G3175" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3176">
@@ -86182,7 +86182,7 @@
         <v>2</v>
       </c>
       <c r="G3176" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3177">
@@ -86209,7 +86209,7 @@
         <v>2</v>
       </c>
       <c r="G3177" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3178">
@@ -86236,7 +86236,7 @@
         <v>2</v>
       </c>
       <c r="G3178" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3179">
@@ -86263,7 +86263,7 @@
         <v>2</v>
       </c>
       <c r="G3179" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3180">
@@ -86290,7 +86290,7 @@
         <v>2</v>
       </c>
       <c r="G3180" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3181">
@@ -86317,7 +86317,7 @@
         <v>2</v>
       </c>
       <c r="G3181" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3182">
@@ -86344,7 +86344,7 @@
         <v>2</v>
       </c>
       <c r="G3182" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3183">
@@ -86371,7 +86371,7 @@
         <v>2</v>
       </c>
       <c r="G3183" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3184">
@@ -86398,7 +86398,7 @@
         <v>2</v>
       </c>
       <c r="G3184" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3185">
@@ -86425,7 +86425,7 @@
         <v>2</v>
       </c>
       <c r="G3185" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3186">
@@ -86452,7 +86452,7 @@
         <v>2</v>
       </c>
       <c r="G3186" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3187">
@@ -86479,7 +86479,7 @@
         <v>2</v>
       </c>
       <c r="G3187" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3188">
@@ -86506,7 +86506,7 @@
         <v>2</v>
       </c>
       <c r="G3188" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3189">
@@ -86533,7 +86533,7 @@
         <v>2</v>
       </c>
       <c r="G3189" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3190">
@@ -86560,7 +86560,7 @@
         <v>2</v>
       </c>
       <c r="G3190" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3191">
@@ -86587,7 +86587,7 @@
         <v>2</v>
       </c>
       <c r="G3191" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3192">
@@ -86614,7 +86614,7 @@
         <v>2</v>
       </c>
       <c r="G3192" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3193">
@@ -86641,7 +86641,7 @@
         <v>2</v>
       </c>
       <c r="G3193" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3194">
@@ -86668,7 +86668,7 @@
         <v>2</v>
       </c>
       <c r="G3194" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3195">
@@ -86695,7 +86695,7 @@
         <v>2</v>
       </c>
       <c r="G3195" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3196">
@@ -86722,7 +86722,7 @@
         <v>2</v>
       </c>
       <c r="G3196" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3197">
@@ -86749,7 +86749,7 @@
         <v>2</v>
       </c>
       <c r="G3197" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3198">
@@ -86776,7 +86776,7 @@
         <v>2</v>
       </c>
       <c r="G3198" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3199">
@@ -86803,7 +86803,7 @@
         <v>2</v>
       </c>
       <c r="G3199" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3200">
@@ -86830,7 +86830,7 @@
         <v>2</v>
       </c>
       <c r="G3200" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3201">
@@ -86857,7 +86857,7 @@
         <v>2</v>
       </c>
       <c r="G3201" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3202">
@@ -86884,7 +86884,7 @@
         <v>2</v>
       </c>
       <c r="G3202" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3203">
@@ -86911,7 +86911,7 @@
         <v>2</v>
       </c>
       <c r="G3203" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3204">
@@ -86938,7 +86938,7 @@
         <v>2</v>
       </c>
       <c r="G3204" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3205">
@@ -86965,7 +86965,7 @@
         <v>2</v>
       </c>
       <c r="G3205" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3206">
@@ -86992,7 +86992,7 @@
         <v>2</v>
       </c>
       <c r="G3206" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3207">
@@ -87019,7 +87019,7 @@
         <v>2</v>
       </c>
       <c r="G3207" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3208">
@@ -87046,7 +87046,7 @@
         <v>2</v>
       </c>
       <c r="G3208" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3209">
@@ -87073,7 +87073,7 @@
         <v>2</v>
       </c>
       <c r="G3209" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3210">
@@ -87100,7 +87100,7 @@
         <v>2</v>
       </c>
       <c r="G3210" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3211">
@@ -87127,7 +87127,7 @@
         <v>2</v>
       </c>
       <c r="G3211" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3212">
@@ -87154,7 +87154,7 @@
         <v>2</v>
       </c>
       <c r="G3212" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3213">
@@ -87181,7 +87181,7 @@
         <v>2</v>
       </c>
       <c r="G3213" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3214">
@@ -87208,7 +87208,7 @@
         <v>2</v>
       </c>
       <c r="G3214" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3215">
@@ -87235,7 +87235,7 @@
         <v>2</v>
       </c>
       <c r="G3215" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3216">
@@ -87262,7 +87262,7 @@
         <v>2</v>
       </c>
       <c r="G3216" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3217">
@@ -87289,7 +87289,7 @@
         <v>2</v>
       </c>
       <c r="G3217" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3218">
@@ -87316,7 +87316,7 @@
         <v>2</v>
       </c>
       <c r="G3218" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3219">
@@ -87343,7 +87343,7 @@
         <v>2</v>
       </c>
       <c r="G3219" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3220">
@@ -87370,7 +87370,7 @@
         <v>2</v>
       </c>
       <c r="G3220" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3221">
@@ -87397,7 +87397,7 @@
         <v>2</v>
       </c>
       <c r="G3221" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3222">
@@ -87424,7 +87424,7 @@
         <v>2</v>
       </c>
       <c r="G3222" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3223">
@@ -87451,7 +87451,7 @@
         <v>2</v>
       </c>
       <c r="G3223" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3224">
@@ -87478,7 +87478,7 @@
         <v>2</v>
       </c>
       <c r="G3224" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3225">
@@ -87505,7 +87505,7 @@
         <v>2</v>
       </c>
       <c r="G3225" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3226">
@@ -87532,7 +87532,7 @@
         <v>2</v>
       </c>
       <c r="G3226" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3227">
@@ -87559,7 +87559,7 @@
         <v>2</v>
       </c>
       <c r="G3227" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3228">
@@ -87586,7 +87586,7 @@
         <v>2</v>
       </c>
       <c r="G3228" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3229">
@@ -87613,7 +87613,7 @@
         <v>2</v>
       </c>
       <c r="G3229" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3230">
@@ -87640,7 +87640,7 @@
         <v>2</v>
       </c>
       <c r="G3230" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3231">
@@ -87667,7 +87667,7 @@
         <v>2</v>
       </c>
       <c r="G3231" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3232">
@@ -87694,7 +87694,7 @@
         <v>2</v>
       </c>
       <c r="G3232" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3233">
@@ -87721,7 +87721,7 @@
         <v>2</v>
       </c>
       <c r="G3233" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3234">
@@ -87748,7 +87748,7 @@
         <v>2</v>
       </c>
       <c r="G3234" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3235">
@@ -87775,7 +87775,7 @@
         <v>2</v>
       </c>
       <c r="G3235" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3236">
@@ -87802,7 +87802,7 @@
         <v>2</v>
       </c>
       <c r="G3236" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3237">
@@ -87829,7 +87829,7 @@
         <v>2</v>
       </c>
       <c r="G3237" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3238">
@@ -87856,7 +87856,7 @@
         <v>2</v>
       </c>
       <c r="G3238" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3239">
@@ -87883,7 +87883,7 @@
         <v>2</v>
       </c>
       <c r="G3239" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3240">
@@ -87910,7 +87910,7 @@
         <v>2</v>
       </c>
       <c r="G3240" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3241">
@@ -87937,7 +87937,7 @@
         <v>2</v>
       </c>
       <c r="G3241" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3242">
@@ -87964,7 +87964,7 @@
         <v>2</v>
       </c>
       <c r="G3242" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3243">
@@ -87991,7 +87991,7 @@
         <v>2</v>
       </c>
       <c r="G3243" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3244">
@@ -88018,7 +88018,7 @@
         <v>2</v>
       </c>
       <c r="G3244" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3245">
@@ -88045,7 +88045,7 @@
         <v>2</v>
       </c>
       <c r="G3245" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3246">
@@ -88072,7 +88072,7 @@
         <v>2</v>
       </c>
       <c r="G3246" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3247">
@@ -88099,7 +88099,7 @@
         <v>2</v>
       </c>
       <c r="G3247" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3248">
@@ -88126,7 +88126,7 @@
         <v>2</v>
       </c>
       <c r="G3248" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3249">
@@ -88153,7 +88153,7 @@
         <v>2</v>
       </c>
       <c r="G3249" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3250">
@@ -88180,7 +88180,7 @@
         <v>2</v>
       </c>
       <c r="G3250" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3251">
@@ -88207,7 +88207,7 @@
         <v>2</v>
       </c>
       <c r="G3251" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3252">
@@ -88234,7 +88234,7 @@
         <v>2</v>
       </c>
       <c r="G3252" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3253">
@@ -88261,7 +88261,7 @@
         <v>2</v>
       </c>
       <c r="G3253" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3254">
@@ -88288,7 +88288,7 @@
         <v>2</v>
       </c>
       <c r="G3254" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3255">
@@ -88315,7 +88315,7 @@
         <v>2</v>
       </c>
       <c r="G3255" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3256">
@@ -88342,7 +88342,7 @@
         <v>2</v>
       </c>
       <c r="G3256" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3257">
@@ -88369,7 +88369,7 @@
         <v>2</v>
       </c>
       <c r="G3257" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3258">
@@ -88396,7 +88396,7 @@
         <v>2</v>
       </c>
       <c r="G3258" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3259">
@@ -88423,7 +88423,7 @@
         <v>2</v>
       </c>
       <c r="G3259" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3260">
@@ -88450,7 +88450,7 @@
         <v>2</v>
       </c>
       <c r="G3260" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3261">
@@ -88477,7 +88477,7 @@
         <v>2</v>
       </c>
       <c r="G3261" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3262">
@@ -88504,7 +88504,7 @@
         <v>2</v>
       </c>
       <c r="G3262" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3263">
@@ -88531,7 +88531,7 @@
         <v>2</v>
       </c>
       <c r="G3263" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3264">
@@ -88558,7 +88558,7 @@
         <v>2</v>
       </c>
       <c r="G3264" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
     <row r="3265">
@@ -88585,7 +88585,7 @@
         <v>2</v>
       </c>
       <c r="G3265" s="2" t="n">
-        <v>46278.46597506487</v>
+        <v>46278.85101434636</v>
       </c>
     </row>
   </sheetData>

</xml_diff>